<commit_message>
walk through module contrasts once for every grouping
</commit_message>
<xml_diff>
--- a/03_Group_comparisons/HRvLR/04_Module_Contrasts/c_data/module_contrasts.xlsx
+++ b/03_Group_comparisons/HRvLR/04_Module_Contrasts/c_data/module_contrasts.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1354" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="290">
   <si>
     <t>sheet</t>
   </si>
@@ -308,16 +308,16 @@
     <t>design</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/01_Design_Contrasts/c_data/design.rds</t>
-  </si>
-  <si>
-    <t>96d863835b9c36a26e09b4706fc4e5e6</t>
+    <t>03_Group_comparisons/HRvLR/01_Design_Contrasts/c_data/design.rds</t>
+  </si>
+  <si>
+    <t>2eec838bcc442e8a2ff1534078b14a38</t>
   </si>
   <si>
     <t>fit</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/02_Protein_Contrasts/c_data/fit.rds</t>
+    <t>03_Group_comparisons/HRvLR/02_Protein_Contrasts/c_data/fit.rds</t>
   </si>
   <si>
     <t>76d83b782ba641782d378b9ae9391e38</t>
@@ -332,7 +332,7 @@
     <t>phenotype</t>
   </si>
   <si>
-    <t>00_Input/phenotype.csv</t>
+    <t>00_Setup/Input/phenotype.csv</t>
   </si>
   <si>
     <t>5a1989db406daa0b70189a9f0df52cf3</t>
@@ -470,6 +470,12 @@
     <t>1.7-17</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>Exact</t>
   </si>
   <si>
@@ -491,6 +497,12 @@
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
     <t>forcats</t>
   </si>
   <si>
@@ -566,6 +578,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>httr</t>
   </si>
   <si>
@@ -584,6 +608,18 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -599,9 +635,6 @@
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>limma</t>
   </si>
   <si>
@@ -653,6 +686,12 @@
     <t>3.1-169</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -731,6 +770,12 @@
     <t>1.3.0</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rootSolve</t>
   </si>
   <si>
@@ -834,6 +879,18 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -11952,7 +12009,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -12216,18 +12273,18 @@
         <v>152</v>
       </c>
       <c r="C24" t="s">
-        <v>153</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>153</v>
+      </c>
+      <c r="B25" t="s">
         <v>154</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>155</v>
-      </c>
-      <c r="C25" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -12312,7 +12369,7 @@
         <v>170</v>
       </c>
       <c r="B33" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="C33" t="s">
         <v>110</v>
@@ -12320,10 +12377,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B34" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C34" t="s">
         <v>110</v>
@@ -12331,10 +12388,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B35" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="C35" t="s">
         <v>110</v>
@@ -12392,7 +12449,7 @@
         <v>184</v>
       </c>
       <c r="C40" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -12436,7 +12493,7 @@
         <v>192</v>
       </c>
       <c r="C44" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -12447,7 +12504,7 @@
         <v>194</v>
       </c>
       <c r="C45" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -12455,7 +12512,7 @@
         <v>195</v>
       </c>
       <c r="B46" t="s">
-        <v>150</v>
+        <v>196</v>
       </c>
       <c r="C46" t="s">
         <v>110</v>
@@ -12463,10 +12520,10 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B47" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C47" t="s">
         <v>110</v>
@@ -12474,10 +12531,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B48" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C48" t="s">
         <v>110</v>
@@ -12485,10 +12542,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B49" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C49" t="s">
         <v>110</v>
@@ -12496,10 +12553,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B50" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="C50" t="s">
         <v>110</v>
@@ -12513,7 +12570,7 @@
         <v>205</v>
       </c>
       <c r="C51" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -12521,7 +12578,7 @@
         <v>206</v>
       </c>
       <c r="B52" t="s">
-        <v>207</v>
+        <v>152</v>
       </c>
       <c r="C52" t="s">
         <v>110</v>
@@ -12529,10 +12586,10 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>207</v>
+      </c>
+      <c r="B53" t="s">
         <v>208</v>
-      </c>
-      <c r="B53" t="s">
-        <v>209</v>
       </c>
       <c r="C53" t="s">
         <v>110</v>
@@ -12540,10 +12597,10 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>209</v>
+      </c>
+      <c r="B54" t="s">
         <v>210</v>
-      </c>
-      <c r="B54" t="s">
-        <v>211</v>
       </c>
       <c r="C54" t="s">
         <v>110</v>
@@ -12551,10 +12608,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>211</v>
+      </c>
+      <c r="B55" t="s">
         <v>212</v>
-      </c>
-      <c r="B55" t="s">
-        <v>213</v>
       </c>
       <c r="C55" t="s">
         <v>110</v>
@@ -12562,10 +12619,10 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
+        <v>213</v>
+      </c>
+      <c r="B56" t="s">
         <v>214</v>
-      </c>
-      <c r="B56" t="s">
-        <v>215</v>
       </c>
       <c r="C56" t="s">
         <v>110</v>
@@ -12573,10 +12630,10 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
+        <v>215</v>
+      </c>
+      <c r="B57" t="s">
         <v>216</v>
-      </c>
-      <c r="B57" t="s">
-        <v>217</v>
       </c>
       <c r="C57" t="s">
         <v>110</v>
@@ -12584,10 +12641,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
+        <v>217</v>
+      </c>
+      <c r="B58" t="s">
         <v>218</v>
-      </c>
-      <c r="B58" t="s">
-        <v>219</v>
       </c>
       <c r="C58" t="s">
         <v>110</v>
@@ -12595,10 +12652,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
+        <v>219</v>
+      </c>
+      <c r="B59" t="s">
         <v>220</v>
-      </c>
-      <c r="B59" t="s">
-        <v>221</v>
       </c>
       <c r="C59" t="s">
         <v>110</v>
@@ -12606,10 +12663,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
+        <v>221</v>
+      </c>
+      <c r="B60" t="s">
         <v>222</v>
-      </c>
-      <c r="B60" t="s">
-        <v>223</v>
       </c>
       <c r="C60" t="s">
         <v>110</v>
@@ -12617,10 +12674,10 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
+        <v>223</v>
+      </c>
+      <c r="B61" t="s">
         <v>224</v>
-      </c>
-      <c r="B61" t="s">
-        <v>225</v>
       </c>
       <c r="C61" t="s">
         <v>110</v>
@@ -12628,10 +12685,10 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
+        <v>225</v>
+      </c>
+      <c r="B62" t="s">
         <v>226</v>
-      </c>
-      <c r="B62" t="s">
-        <v>227</v>
       </c>
       <c r="C62" t="s">
         <v>110</v>
@@ -12639,10 +12696,10 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
+        <v>227</v>
+      </c>
+      <c r="B63" t="s">
         <v>228</v>
-      </c>
-      <c r="B63" t="s">
-        <v>229</v>
       </c>
       <c r="C63" t="s">
         <v>110</v>
@@ -12650,10 +12707,10 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
+        <v>229</v>
+      </c>
+      <c r="B64" t="s">
         <v>230</v>
-      </c>
-      <c r="B64" t="s">
-        <v>231</v>
       </c>
       <c r="C64" t="s">
         <v>110</v>
@@ -12661,10 +12718,10 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
+        <v>231</v>
+      </c>
+      <c r="B65" t="s">
         <v>232</v>
-      </c>
-      <c r="B65" t="s">
-        <v>233</v>
       </c>
       <c r="C65" t="s">
         <v>110</v>
@@ -12672,21 +12729,21 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
+        <v>233</v>
+      </c>
+      <c r="B66" t="s">
         <v>234</v>
       </c>
-      <c r="B66" t="s">
-        <v>235</v>
-      </c>
       <c r="C66" t="s">
-        <v>153</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
+        <v>235</v>
+      </c>
+      <c r="B67" t="s">
         <v>236</v>
-      </c>
-      <c r="B67" t="s">
-        <v>237</v>
       </c>
       <c r="C67" t="s">
         <v>110</v>
@@ -12694,10 +12751,10 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
+        <v>237</v>
+      </c>
+      <c r="B68" t="s">
         <v>238</v>
-      </c>
-      <c r="B68" t="s">
-        <v>239</v>
       </c>
       <c r="C68" t="s">
         <v>110</v>
@@ -12705,10 +12762,10 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
+        <v>239</v>
+      </c>
+      <c r="B69" t="s">
         <v>240</v>
-      </c>
-      <c r="B69" t="s">
-        <v>241</v>
       </c>
       <c r="C69" t="s">
         <v>110</v>
@@ -12716,21 +12773,21 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
+        <v>241</v>
+      </c>
+      <c r="B70" t="s">
         <v>242</v>
       </c>
-      <c r="B70" t="s">
-        <v>243</v>
-      </c>
       <c r="C70" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
+        <v>243</v>
+      </c>
+      <c r="B71" t="s">
         <v>244</v>
-      </c>
-      <c r="B71" t="s">
-        <v>245</v>
       </c>
       <c r="C71" t="s">
         <v>110</v>
@@ -12738,10 +12795,10 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
+        <v>245</v>
+      </c>
+      <c r="B72" t="s">
         <v>246</v>
-      </c>
-      <c r="B72" t="s">
-        <v>247</v>
       </c>
       <c r="C72" t="s">
         <v>110</v>
@@ -12749,21 +12806,21 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
+        <v>247</v>
+      </c>
+      <c r="B73" t="s">
         <v>248</v>
       </c>
-      <c r="B73" t="s">
-        <v>249</v>
-      </c>
       <c r="C73" t="s">
-        <v>110</v>
+        <v>155</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
+        <v>249</v>
+      </c>
+      <c r="B74" t="s">
         <v>250</v>
-      </c>
-      <c r="B74" t="s">
-        <v>251</v>
       </c>
       <c r="C74" t="s">
         <v>110</v>
@@ -12771,10 +12828,10 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
+        <v>251</v>
+      </c>
+      <c r="B75" t="s">
         <v>252</v>
-      </c>
-      <c r="B75" t="s">
-        <v>253</v>
       </c>
       <c r="C75" t="s">
         <v>110</v>
@@ -12782,10 +12839,10 @@
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
+        <v>253</v>
+      </c>
+      <c r="B76" t="s">
         <v>254</v>
-      </c>
-      <c r="B76" t="s">
-        <v>255</v>
       </c>
       <c r="C76" t="s">
         <v>110</v>
@@ -12793,10 +12850,10 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
+        <v>255</v>
+      </c>
+      <c r="B77" t="s">
         <v>256</v>
-      </c>
-      <c r="B77" t="s">
-        <v>257</v>
       </c>
       <c r="C77" t="s">
         <v>110</v>
@@ -12804,21 +12861,21 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
+        <v>257</v>
+      </c>
+      <c r="B78" t="s">
         <v>258</v>
       </c>
-      <c r="B78" t="s">
-        <v>259</v>
-      </c>
       <c r="C78" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
+        <v>259</v>
+      </c>
+      <c r="B79" t="s">
         <v>260</v>
-      </c>
-      <c r="B79" t="s">
-        <v>261</v>
       </c>
       <c r="C79" t="s">
         <v>110</v>
@@ -12826,10 +12883,10 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
+        <v>261</v>
+      </c>
+      <c r="B80" t="s">
         <v>262</v>
-      </c>
-      <c r="B80" t="s">
-        <v>146</v>
       </c>
       <c r="C80" t="s">
         <v>110</v>
@@ -12876,6 +12933,116 @@
         <v>270</v>
       </c>
       <c r="C84" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" t="s">
+        <v>271</v>
+      </c>
+      <c r="B85" t="s">
+        <v>272</v>
+      </c>
+      <c r="C85" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" t="s">
+        <v>273</v>
+      </c>
+      <c r="B86" t="s">
+        <v>274</v>
+      </c>
+      <c r="C86" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" t="s">
+        <v>275</v>
+      </c>
+      <c r="B87" t="s">
+        <v>276</v>
+      </c>
+      <c r="C87" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" t="s">
+        <v>277</v>
+      </c>
+      <c r="B88" t="s">
+        <v>146</v>
+      </c>
+      <c r="C88" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" t="s">
+        <v>278</v>
+      </c>
+      <c r="B89" t="s">
+        <v>279</v>
+      </c>
+      <c r="C89" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" t="s">
+        <v>280</v>
+      </c>
+      <c r="B90" t="s">
+        <v>281</v>
+      </c>
+      <c r="C90" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3">
+      <c r="A91" t="s">
+        <v>282</v>
+      </c>
+      <c r="B91" t="s">
+        <v>283</v>
+      </c>
+      <c r="C91" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" t="s">
+        <v>284</v>
+      </c>
+      <c r="B92" t="s">
+        <v>285</v>
+      </c>
+      <c r="C92" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3">
+      <c r="A93" t="s">
+        <v>286</v>
+      </c>
+      <c r="B93" t="s">
+        <v>287</v>
+      </c>
+      <c r="C93" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" t="s">
+        <v>288</v>
+      </c>
+      <c r="B94" t="s">
+        <v>289</v>
+      </c>
+      <c r="C94" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>